<commit_message>
Update scraped data [2026-08-30]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="459">
   <si>
     <t>date</t>
   </si>
@@ -1389,6 +1389,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/canada/canadian-premier-league/, /football/egypt/premier-league/, /football/el-salvador/primera-division/, /football/estonia/esiliiga/, /football/guatemala/liga-nacional/, /football/iceland/division-1/, /football/northern-ireland/nifl-premiership/, /football/paraguay/copa-de-primera/, /football/peru/liga-1/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3b99dc8965474858f4d1d889b4626609aefa7f30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/egypt/premier-league/, /football/greece/super-league/, /football/ireland/division-1/, /football/northern-ireland/nifl-premiership/, /football/sweden/superettan/, /football/switzerland/super-league/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -11985,6 +11991,47 @@
         <v>457</v>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B252" t="s">
+        <v>458</v>
+      </c>
+      <c r="C252" t="s">
+        <v>31</v>
+      </c>
+      <c r="D252" t="n">
+        <v>312.957677892844</v>
+      </c>
+      <c r="E252" t="n">
+        <v>74</v>
+      </c>
+      <c r="F252" t="n">
+        <v>0</v>
+      </c>
+      <c r="G252" t="n">
+        <v>413</v>
+      </c>
+      <c r="H252" t="n">
+        <v>345</v>
+      </c>
+      <c r="I252" t="n">
+        <v>68</v>
+      </c>
+      <c r="J252" t="n">
+        <v>211</v>
+      </c>
+      <c r="K252" t="n">
+        <v>7662</v>
+      </c>
+      <c r="L252" t="n">
+        <v>29</v>
+      </c>
+      <c r="M252" t="s">
+        <v>459</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-17]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="461">
   <si>
     <t>date</t>
   </si>
@@ -1395,6 +1395,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/egypt/premier-league/, /football/greece/super-league/, /football/ireland/division-1/, /football/northern-ireland/nifl-premiership/, /football/sweden/superettan/, /football/switzerland/super-league/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6addcf3b0e551def84e9c5d095076040a25af789</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/costa-rica/liga-de-ascenso/, /football/finland/ykkosliiga/, /football/northern-ireland/nifl-premiership/</t>
   </si>
 </sst>
 </file>
@@ -12032,6 +12038,47 @@
         <v>459</v>
       </c>
     </row>
+    <row r="253">
+      <c r="A253" s="1" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B253" t="s">
+        <v>460</v>
+      </c>
+      <c r="C253" t="s">
+        <v>31</v>
+      </c>
+      <c r="D253" t="n">
+        <v>283.754804599285</v>
+      </c>
+      <c r="E253" t="n">
+        <v>66</v>
+      </c>
+      <c r="F253" t="n">
+        <v>0</v>
+      </c>
+      <c r="G253" t="n">
+        <v>427</v>
+      </c>
+      <c r="H253" t="n">
+        <v>379</v>
+      </c>
+      <c r="I253" t="n">
+        <v>48</v>
+      </c>
+      <c r="J253" t="n">
+        <v>255</v>
+      </c>
+      <c r="K253" t="n">
+        <v>7644</v>
+      </c>
+      <c r="L253" t="n">
+        <v>25</v>
+      </c>
+      <c r="M253" t="s">
+        <v>461</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-18]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="463">
   <si>
     <t>date</t>
   </si>
@@ -1401,6 +1401,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/costa-rica/liga-de-ascenso/, /football/finland/ykkosliiga/, /football/northern-ireland/nifl-premiership/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e7a4c721380ad05592e2d4e16b6bc9d5f8aa118c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/finland/ykkosliiga/</t>
   </si>
 </sst>
 </file>
@@ -12079,6 +12085,47 @@
         <v>461</v>
       </c>
     </row>
+    <row r="254">
+      <c r="A254" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B254" t="s">
+        <v>462</v>
+      </c>
+      <c r="C254" t="s">
+        <v>31</v>
+      </c>
+      <c r="D254" t="n">
+        <v>323.261201198896</v>
+      </c>
+      <c r="E254" t="n">
+        <v>75</v>
+      </c>
+      <c r="F254" t="n">
+        <v>0</v>
+      </c>
+      <c r="G254" t="n">
+        <v>505</v>
+      </c>
+      <c r="H254" t="n">
+        <v>242</v>
+      </c>
+      <c r="I254" t="n">
+        <v>263</v>
+      </c>
+      <c r="J254" t="n">
+        <v>78</v>
+      </c>
+      <c r="K254" t="n">
+        <v>8635</v>
+      </c>
+      <c r="L254" t="n">
+        <v>33</v>
+      </c>
+      <c r="M254" t="s">
+        <v>463</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-19]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="467">
   <si>
     <t>date</t>
   </si>
@@ -1413,6 +1413,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/finland/ykkosliiga/, /football/ireland/premier-division/, /football/uruguay/segunda-division/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b04876cb24125636d8988905b463da40c88f85ad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/ireland/division-1/, /football/netherlands/eerste-divisie/, /football/northern-ireland/nifl-premiership/, /football/romania/superliga/, /football/uruguay/segunda-division/, /football/venezuela/liga-futve/</t>
   </si>
 </sst>
 </file>
@@ -12173,6 +12179,47 @@
         <v>465</v>
       </c>
     </row>
+    <row r="256">
+      <c r="A256" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B256" t="s">
+        <v>466</v>
+      </c>
+      <c r="C256" t="s">
+        <v>31</v>
+      </c>
+      <c r="D256" t="n">
+        <v>309.971255501111</v>
+      </c>
+      <c r="E256" t="n">
+        <v>66</v>
+      </c>
+      <c r="F256" t="n">
+        <v>0</v>
+      </c>
+      <c r="G256" t="n">
+        <v>295</v>
+      </c>
+      <c r="H256" t="n">
+        <v>117</v>
+      </c>
+      <c r="I256" t="n">
+        <v>178</v>
+      </c>
+      <c r="J256" t="n">
+        <v>132</v>
+      </c>
+      <c r="K256" t="n">
+        <v>7601</v>
+      </c>
+      <c r="L256" t="n">
+        <v>21</v>
+      </c>
+      <c r="M256" t="s">
+        <v>467</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-20]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="469">
   <si>
     <t>date</t>
   </si>
@@ -1419,6 +1419,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/ireland/division-1/, /football/netherlands/eerste-divisie/, /football/northern-ireland/nifl-premiership/, /football/romania/superliga/, /football/uruguay/segunda-division/, /football/venezuela/liga-futve/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bf5be29f1a874ee8837eb01cdffe1ff0786c51aa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/colombia/primera-b/, /football/finland/ykkosliiga/, /football/netherlands/eerste-divisie/, /football/northern-ireland/nifl-premiership/</t>
   </si>
 </sst>
 </file>
@@ -12220,6 +12226,47 @@
         <v>467</v>
       </c>
     </row>
+    <row r="257">
+      <c r="A257" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B257" t="s">
+        <v>468</v>
+      </c>
+      <c r="C257" t="s">
+        <v>31</v>
+      </c>
+      <c r="D257" t="n">
+        <v>242.538366731008</v>
+      </c>
+      <c r="E257" t="n">
+        <v>57</v>
+      </c>
+      <c r="F257" t="n">
+        <v>0</v>
+      </c>
+      <c r="G257" t="n">
+        <v>250</v>
+      </c>
+      <c r="H257" t="n">
+        <v>106</v>
+      </c>
+      <c r="I257" t="n">
+        <v>144</v>
+      </c>
+      <c r="J257" t="n">
+        <v>57</v>
+      </c>
+      <c r="K257" t="n">
+        <v>6359</v>
+      </c>
+      <c r="L257" t="n">
+        <v>19</v>
+      </c>
+      <c r="M257" t="s">
+        <v>469</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-21]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="473">
   <si>
     <t>date</t>
   </si>
@@ -1431,6 +1431,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/colombia/primera-a/, /football/mexico/liga-de-expansion-mx/, /football/northern-ireland/nifl-premiership/, /football/romania/superliga/, /football/venezuela/liga-futve/, /football/venezuela/liga-futve-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">488b6e9ce9af5a7b44c1968339a5f41fe00847c2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/estonia/meistriliiga/, /football/kazakhstan/premier-league/, /football/northern-ireland/nifl-premiership/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -12314,6 +12320,47 @@
         <v>471</v>
       </c>
     </row>
+    <row r="259">
+      <c r="A259" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B259" t="s">
+        <v>472</v>
+      </c>
+      <c r="C259" t="s">
+        <v>31</v>
+      </c>
+      <c r="D259" t="n">
+        <v>184.427565085888</v>
+      </c>
+      <c r="E259" t="n">
+        <v>30</v>
+      </c>
+      <c r="F259" t="n">
+        <v>0</v>
+      </c>
+      <c r="G259" t="n">
+        <v>218</v>
+      </c>
+      <c r="H259" t="n">
+        <v>144</v>
+      </c>
+      <c r="I259" t="n">
+        <v>74</v>
+      </c>
+      <c r="J259" t="n">
+        <v>45</v>
+      </c>
+      <c r="K259" t="n">
+        <v>4491</v>
+      </c>
+      <c r="L259" t="n">
+        <v>14</v>
+      </c>
+      <c r="M259" t="s">
+        <v>473</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-22]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="475">
   <si>
     <t>date</t>
   </si>
@@ -1437,6 +1437,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/meistriliiga/, /football/kazakhstan/premier-league/, /football/northern-ireland/nifl-premiership/, /football/usa/usl-championship/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d29dd8c9e9070fad933a6731d6ea7a4482a29fa1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/estonia/meistriliiga/, /football/finland/ykkosliiga/, /football/kazakhstan/premier-league/, /football/northern-ireland/nifl-premiership/, /football/poland/ekstraklasa/</t>
   </si>
 </sst>
 </file>
@@ -12361,6 +12367,47 @@
         <v>473</v>
       </c>
     </row>
+    <row r="260">
+      <c r="A260" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B260" t="s">
+        <v>474</v>
+      </c>
+      <c r="C260" t="s">
+        <v>31</v>
+      </c>
+      <c r="D260" t="n">
+        <v>233.026022803783</v>
+      </c>
+      <c r="E260" t="n">
+        <v>36</v>
+      </c>
+      <c r="F260" t="n">
+        <v>0</v>
+      </c>
+      <c r="G260" t="n">
+        <v>282</v>
+      </c>
+      <c r="H260" t="n">
+        <v>151</v>
+      </c>
+      <c r="I260" t="n">
+        <v>131</v>
+      </c>
+      <c r="J260" t="n">
+        <v>6</v>
+      </c>
+      <c r="K260" t="n">
+        <v>5191</v>
+      </c>
+      <c r="L260" t="n">
+        <v>17</v>
+      </c>
+      <c r="M260" t="s">
+        <v>475</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-23]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="477">
   <si>
     <t>date</t>
   </si>
@@ -1443,6 +1443,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/meistriliiga/, /football/finland/ykkosliiga/, /football/kazakhstan/premier-league/, /football/northern-ireland/nifl-premiership/, /football/poland/ekstraklasa/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">91438f3d59d7936d3aee86ce10690e845f85174b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/canada/canadian-premier-league/, /football/colombia/primera-a/, /football/el-salvador/primera-division/, /football/guatemala/liga-nacional/, /football/romania/superliga/, /football/slovenia/prva-liga/</t>
   </si>
 </sst>
 </file>
@@ -12408,6 +12414,47 @@
         <v>475</v>
       </c>
     </row>
+    <row r="261">
+      <c r="A261" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B261" t="s">
+        <v>476</v>
+      </c>
+      <c r="C261" t="s">
+        <v>31</v>
+      </c>
+      <c r="D261" t="n">
+        <v>245.448450366656</v>
+      </c>
+      <c r="E261" t="n">
+        <v>30</v>
+      </c>
+      <c r="F261" t="n">
+        <v>0</v>
+      </c>
+      <c r="G261" t="n">
+        <v>223</v>
+      </c>
+      <c r="H261" t="n">
+        <v>72</v>
+      </c>
+      <c r="I261" t="n">
+        <v>151</v>
+      </c>
+      <c r="J261" t="n">
+        <v>1</v>
+      </c>
+      <c r="K261" t="n">
+        <v>4156</v>
+      </c>
+      <c r="L261" t="n">
+        <v>12</v>
+      </c>
+      <c r="M261" t="s">
+        <v>477</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-24]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="481">
   <si>
     <t>date</t>
   </si>
@@ -1455,6 +1455,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/canada/canadian-premier-league/, /football/ecuador/serie-b/, /football/estonia/meistriliiga/, /football/finland/ykkosliiga/, /football/guatemala/liga-nacional/, /football/northern-ireland/nifl-premiership/, /football/paraguay/copa-de-primera/, /football/romania/superliga/, /football/slovakia/nike-liga/, /football/slovakia/nike-liga/, /football/slovenia/prva-liga/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6fc93a69ed856d7072dfda89c12306cb9c69d688</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/ecuador/serie-b/, /football/el-salvador/primera-division/, /football/guatemala/liga-nacional/, /football/romania/superliga/, /football/slovakia/nike-liga/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -12502,6 +12508,47 @@
         <v>479</v>
       </c>
     </row>
+    <row r="263">
+      <c r="A263" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B263" t="s">
+        <v>480</v>
+      </c>
+      <c r="C263" t="s">
+        <v>31</v>
+      </c>
+      <c r="D263" t="n">
+        <v>219.441783471902</v>
+      </c>
+      <c r="E263" t="n">
+        <v>34</v>
+      </c>
+      <c r="F263" t="n">
+        <v>0</v>
+      </c>
+      <c r="G263" t="n">
+        <v>270</v>
+      </c>
+      <c r="H263" t="n">
+        <v>76</v>
+      </c>
+      <c r="I263" t="n">
+        <v>194</v>
+      </c>
+      <c r="J263" t="n">
+        <v>4</v>
+      </c>
+      <c r="K263" t="n">
+        <v>4944</v>
+      </c>
+      <c r="L263" t="n">
+        <v>11</v>
+      </c>
+      <c r="M263" t="s">
+        <v>481</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-25]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="485">
   <si>
     <t>date</t>
   </si>
@@ -1467,6 +1467,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/canada/canadian-premier-league/, /football/colombia/primera-a/, /football/estonia/meistriliiga/, /football/paraguay/copa-de-primera/, /football/paraguay/division-intermedia/, /football/romania/superliga/, /football/slovenia/prva-liga/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9cdf052efce6cb079715e88f46892e3a739560c5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/bosnia-and-herzegovina/prva-liga-fbih/, /football/el-salvador/primera-division/, /football/finland/ykkosliiga/, /football/kazakhstan/premier-league/, /football/romania/superliga/, /football/slovakia/nike-liga/, /football/slovenia/prva-liga/, /football/ukraine/premier-league/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -12596,6 +12602,47 @@
         <v>483</v>
       </c>
     </row>
+    <row r="265">
+      <c r="A265" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B265" t="s">
+        <v>484</v>
+      </c>
+      <c r="C265" t="s">
+        <v>31</v>
+      </c>
+      <c r="D265" t="n">
+        <v>314.776300156116</v>
+      </c>
+      <c r="E265" t="n">
+        <v>40</v>
+      </c>
+      <c r="F265" t="n">
+        <v>0</v>
+      </c>
+      <c r="G265" t="n">
+        <v>290</v>
+      </c>
+      <c r="H265" t="n">
+        <v>84</v>
+      </c>
+      <c r="I265" t="n">
+        <v>206</v>
+      </c>
+      <c r="J265" t="n">
+        <v>4</v>
+      </c>
+      <c r="K265" t="n">
+        <v>5267</v>
+      </c>
+      <c r="L265" t="n">
+        <v>21</v>
+      </c>
+      <c r="M265" t="s">
+        <v>485</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-26]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="485">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="487">
   <si>
     <t>date</t>
   </si>
@@ -1473,6 +1473,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/bosnia-and-herzegovina/prva-liga-fbih/, /football/el-salvador/primera-division/, /football/finland/ykkosliiga/, /football/kazakhstan/premier-league/, /football/romania/superliga/, /football/slovakia/nike-liga/, /football/slovenia/prva-liga/, /football/ukraine/premier-league/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">73a76631f6c634bc6a1c52ad00f856ff87abfea8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/colombia/primera-a/, /football/colombia/primera-b/, /football/estonia/meistriliiga/, /football/ireland/division-1/, /football/paraguay/copa-de-primera/, /football/romania/superliga/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -12643,6 +12649,47 @@
         <v>485</v>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B266" t="s">
+        <v>486</v>
+      </c>
+      <c r="C266" t="s">
+        <v>31</v>
+      </c>
+      <c r="D266" t="n">
+        <v>339.635323941708</v>
+      </c>
+      <c r="E266" t="n">
+        <v>49</v>
+      </c>
+      <c r="F266" t="n">
+        <v>0</v>
+      </c>
+      <c r="G266" t="n">
+        <v>332</v>
+      </c>
+      <c r="H266" t="n">
+        <v>133</v>
+      </c>
+      <c r="I266" t="n">
+        <v>199</v>
+      </c>
+      <c r="J266" t="n">
+        <v>2</v>
+      </c>
+      <c r="K266" t="n">
+        <v>5973</v>
+      </c>
+      <c r="L266" t="n">
+        <v>25</v>
+      </c>
+      <c r="M266" t="s">
+        <v>487</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-27]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="491">
   <si>
     <t>date</t>
   </si>
@@ -1485,6 +1485,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/costa-rica/liga-de-ascenso/, /football/slovenia/prva-liga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5b2588dc448dac18ad736500f1d8aa808019b146</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/brazil/serie-a-betano/, /football/colombia/primera-b/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/northern-ireland/nifl-premiership/, /football/poland/division-1/, /football/poland/division-1/</t>
   </si>
 </sst>
 </file>
@@ -12737,6 +12743,47 @@
         <v>489</v>
       </c>
     </row>
+    <row r="268">
+      <c r="A268" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B268" t="s">
+        <v>490</v>
+      </c>
+      <c r="C268" t="s">
+        <v>31</v>
+      </c>
+      <c r="D268" t="n">
+        <v>236.712737429142</v>
+      </c>
+      <c r="E268" t="n">
+        <v>38</v>
+      </c>
+      <c r="F268" t="n">
+        <v>0</v>
+      </c>
+      <c r="G268" t="n">
+        <v>301</v>
+      </c>
+      <c r="H268" t="n">
+        <v>112</v>
+      </c>
+      <c r="I268" t="n">
+        <v>189</v>
+      </c>
+      <c r="J268" t="n">
+        <v>37</v>
+      </c>
+      <c r="K268" t="n">
+        <v>5050</v>
+      </c>
+      <c r="L268" t="n">
+        <v>18</v>
+      </c>
+      <c r="M268" t="s">
+        <v>491</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-28]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="493">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="495">
   <si>
     <t>date</t>
   </si>
@@ -1497,6 +1497,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/argentina/primera-nacional/, /football/ireland/division-1/, /football/paraguay/copa-de-primera/, /football/poland/ekstraklasa/, /football/slovenia/prva-liga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6766472afed582c52f4f3685edf197b7fded469f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/estonia/meistriliiga/, /football/estonia/meistriliiga/, /football/kazakhstan/premier-league/, /football/northern-ireland/nifl-premiership/</t>
   </si>
 </sst>
 </file>
@@ -12831,6 +12837,47 @@
         <v>493</v>
       </c>
     </row>
+    <row r="270">
+      <c r="A270" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B270" t="s">
+        <v>494</v>
+      </c>
+      <c r="C270" t="s">
+        <v>31</v>
+      </c>
+      <c r="D270" t="n">
+        <v>214.379126723607</v>
+      </c>
+      <c r="E270" t="n">
+        <v>33</v>
+      </c>
+      <c r="F270" t="n">
+        <v>0</v>
+      </c>
+      <c r="G270" t="n">
+        <v>299</v>
+      </c>
+      <c r="H270" t="n">
+        <v>123</v>
+      </c>
+      <c r="I270" t="n">
+        <v>176</v>
+      </c>
+      <c r="J270" t="n">
+        <v>14</v>
+      </c>
+      <c r="K270" t="n">
+        <v>4815</v>
+      </c>
+      <c r="L270" t="n">
+        <v>13</v>
+      </c>
+      <c r="M270" t="s">
+        <v>495</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-29]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="497">
   <si>
     <t>date</t>
   </si>
@@ -1503,6 +1503,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/estonia/meistriliiga/, /football/estonia/meistriliiga/, /football/kazakhstan/premier-league/, /football/northern-ireland/nifl-premiership/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">49a1de4d6b2fb0f4566ddae0ef7714ff43d9d661</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/colombia/primera-b/, /football/kazakhstan/premier-league/, /football/northern-ireland/nifl-premiership/, /football/paraguay/copa-de-primera/, /football/peru/liga-1/, /football/poland/ekstraklasa/, /football/slovenia/prva-liga/, /football/ukraine/premier-league/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -12878,6 +12884,47 @@
         <v>495</v>
       </c>
     </row>
+    <row r="271">
+      <c r="A271" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B271" t="s">
+        <v>496</v>
+      </c>
+      <c r="C271" t="s">
+        <v>31</v>
+      </c>
+      <c r="D271" t="n">
+        <v>210.896491126219</v>
+      </c>
+      <c r="E271" t="n">
+        <v>40</v>
+      </c>
+      <c r="F271" t="n">
+        <v>0</v>
+      </c>
+      <c r="G271" t="n">
+        <v>384</v>
+      </c>
+      <c r="H271" t="n">
+        <v>127</v>
+      </c>
+      <c r="I271" t="n">
+        <v>257</v>
+      </c>
+      <c r="J271" t="n">
+        <v>9</v>
+      </c>
+      <c r="K271" t="n">
+        <v>5833</v>
+      </c>
+      <c r="L271" t="n">
+        <v>18</v>
+      </c>
+      <c r="M271" t="s">
+        <v>497</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-09-30]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="503">
   <si>
     <t>date</t>
   </si>
@@ -1521,6 +1521,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/canada/canadian-premier-league/, /football/chile/liga-de-ascenso/, /football/estonia/meistriliiga/, /football/guatemala/liga-nacional/, /football/mexico/liga-de-expansion-mx/, /football/paraguay/copa-de-primera/, /football/poland/division-1/, /football/slovenia/prva-liga/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3dd761484bc7d4db897236a6b756be81ee23c2b0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/estonia/meistriliiga/, /football/northern-ireland/nifl-premiership/, /football/peru/liga-1/, /football/poland/ekstraklasa/, /football/poland/division-1/, /football/romania/liga-2/, /football/ukraine/premier-league/, /football/uruguay/liga-auf-uruguaya/</t>
   </si>
 </sst>
 </file>
@@ -13019,6 +13025,47 @@
         <v>501</v>
       </c>
     </row>
+    <row r="274">
+      <c r="A274" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B274" t="s">
+        <v>502</v>
+      </c>
+      <c r="C274" t="s">
+        <v>31</v>
+      </c>
+      <c r="D274" t="n">
+        <v>201.0618810455</v>
+      </c>
+      <c r="E274" t="n">
+        <v>41</v>
+      </c>
+      <c r="F274" t="n">
+        <v>0</v>
+      </c>
+      <c r="G274" t="n">
+        <v>361</v>
+      </c>
+      <c r="H274" t="n">
+        <v>116</v>
+      </c>
+      <c r="I274" t="n">
+        <v>245</v>
+      </c>
+      <c r="J274" t="n">
+        <v>0</v>
+      </c>
+      <c r="K274" t="n">
+        <v>5750</v>
+      </c>
+      <c r="L274" t="n">
+        <v>19</v>
+      </c>
+      <c r="M274" t="s">
+        <v>503</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-01]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="505">
   <si>
     <t>date</t>
   </si>
@@ -1527,6 +1527,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/estonia/meistriliiga/, /football/northern-ireland/nifl-premiership/, /football/peru/liga-1/, /football/poland/ekstraklasa/, /football/poland/division-1/, /football/romania/liga-2/, /football/ukraine/premier-league/, /football/uruguay/liga-auf-uruguaya/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8d29ab56e3eb5099cdfef87d0813fcedb793435d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/colombia/primera-b/, /football/paraguay/copa-de-primera/, /football/poland/division-1/, /football/romania/liga-2/, /football/romania/liga-2/, /football/ukraine/premier-league/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -13066,6 +13072,47 @@
         <v>503</v>
       </c>
     </row>
+    <row r="275">
+      <c r="A275" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B275" t="s">
+        <v>504</v>
+      </c>
+      <c r="C275" t="s">
+        <v>31</v>
+      </c>
+      <c r="D275" t="n">
+        <v>260.790433597565</v>
+      </c>
+      <c r="E275" t="n">
+        <v>41</v>
+      </c>
+      <c r="F275" t="n">
+        <v>0</v>
+      </c>
+      <c r="G275" t="n">
+        <v>383</v>
+      </c>
+      <c r="H275" t="n">
+        <v>120</v>
+      </c>
+      <c r="I275" t="n">
+        <v>263</v>
+      </c>
+      <c r="J275" t="n">
+        <v>0</v>
+      </c>
+      <c r="K275" t="n">
+        <v>5767</v>
+      </c>
+      <c r="L275" t="n">
+        <v>20</v>
+      </c>
+      <c r="M275" t="s">
+        <v>505</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-03]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="510">
   <si>
     <t>date</t>
   </si>
@@ -1542,6 +1542,12 @@
   </si>
   <si>
     <t xml:space="preserve">b086b8c051c19de0cde841b0269fb3a0d2fabed5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d9d1ebd2e707f59b78b557a50ddf5f5692c47212</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/colombia/primera-a/, /football/ecuador/serie-b/, /football/el-salvador/primera-division/, /football/estonia/meistriliiga/, /football/kazakhstan/premier-league/, /football/mexico/liga-mx/, /football/paraguay/copa-de-primera/, /football/romania/superliga/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -13204,6 +13210,47 @@
         <v>184</v>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" s="1" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B278" t="s">
+        <v>509</v>
+      </c>
+      <c r="C278" t="s">
+        <v>31</v>
+      </c>
+      <c r="D278" t="n">
+        <v>252.162192988396</v>
+      </c>
+      <c r="E278" t="n">
+        <v>57</v>
+      </c>
+      <c r="F278" t="n">
+        <v>0</v>
+      </c>
+      <c r="G278" t="n">
+        <v>429</v>
+      </c>
+      <c r="H278" t="n">
+        <v>63</v>
+      </c>
+      <c r="I278" t="n">
+        <v>366</v>
+      </c>
+      <c r="J278" t="n">
+        <v>13</v>
+      </c>
+      <c r="K278" t="n">
+        <v>7821</v>
+      </c>
+      <c r="L278" t="n">
+        <v>25</v>
+      </c>
+      <c r="M278" t="s">
+        <v>510</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-04]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="516">
   <si>
     <t>date</t>
   </si>
@@ -1560,6 +1560,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/canada/canadian-premier-league/, /football/colombia/primera-a/, /football/romania/superliga/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42498ca227708b7fad19e5e1d462d8e83815fe17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/belgium/challenger-pro-league/, /football/bulgaria/vtora-liga/, /football/costa-rica/liga-de-ascenso/, /football/ecuador/serie-b/, /football/kazakhstan/premier-league/, /football/paraguay/division-intermedia/, /football/poland/division-1/, /football/romania/superliga/, /football/romania/liga-2/, /football/ukraine/premier-league/</t>
   </si>
 </sst>
 </file>
@@ -13345,6 +13351,47 @@
         <v>514</v>
       </c>
     </row>
+    <row r="281">
+      <c r="A281" s="1" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B281" t="s">
+        <v>515</v>
+      </c>
+      <c r="C281" t="s">
+        <v>31</v>
+      </c>
+      <c r="D281" t="n">
+        <v>301.685932131608</v>
+      </c>
+      <c r="E281" t="n">
+        <v>62</v>
+      </c>
+      <c r="F281" t="n">
+        <v>0</v>
+      </c>
+      <c r="G281" t="n">
+        <v>457</v>
+      </c>
+      <c r="H281" t="n">
+        <v>120</v>
+      </c>
+      <c r="I281" t="n">
+        <v>337</v>
+      </c>
+      <c r="J281" t="n">
+        <v>39</v>
+      </c>
+      <c r="K281" t="n">
+        <v>8469</v>
+      </c>
+      <c r="L281" t="n">
+        <v>33</v>
+      </c>
+      <c r="M281" t="s">
+        <v>516</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-05]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="520">
   <si>
     <t>date</t>
   </si>
@@ -1572,6 +1572,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/belgium/challenger-pro-league/, /football/bulgaria/vtora-liga/, /football/canada/canadian-premier-league/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/paraguay/division-intermedia/, /football/poland/division-1/, /football/romania/liga-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cdaf3da4f6fa118662fea4adb7a289d4be2c0273</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/belgium/jupiler-pro-league/, /football/bulgaria/vtora-liga/, /football/iraq/stars-league/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/romania/superliga/, /football/romania/liga-2/</t>
   </si>
 </sst>
 </file>
@@ -13439,6 +13445,47 @@
         <v>518</v>
       </c>
     </row>
+    <row r="283">
+      <c r="A283" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B283" t="s">
+        <v>519</v>
+      </c>
+      <c r="C283" t="s">
+        <v>31</v>
+      </c>
+      <c r="D283" t="n">
+        <v>271.50768515269</v>
+      </c>
+      <c r="E283" t="n">
+        <v>54</v>
+      </c>
+      <c r="F283" t="n">
+        <v>0</v>
+      </c>
+      <c r="G283" t="n">
+        <v>497</v>
+      </c>
+      <c r="H283" t="n">
+        <v>115</v>
+      </c>
+      <c r="I283" t="n">
+        <v>382</v>
+      </c>
+      <c r="J283" t="n">
+        <v>28</v>
+      </c>
+      <c r="K283" t="n">
+        <v>7486</v>
+      </c>
+      <c r="L283" t="n">
+        <v>23</v>
+      </c>
+      <c r="M283" t="s">
+        <v>520</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-06]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="522">
   <si>
     <t>date</t>
   </si>
@@ -1578,6 +1578,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/belgium/jupiler-pro-league/, /football/bulgaria/vtora-liga/, /football/iraq/stars-league/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/romania/superliga/, /football/romania/liga-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">99c1746ee6237b094159fb6b34b2352a600b6474</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/belgium/jupiler-pro-league/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/peru/liga-2/, /football/romania/liga-2/</t>
   </si>
 </sst>
 </file>
@@ -13486,6 +13492,47 @@
         <v>520</v>
       </c>
     </row>
+    <row r="284">
+      <c r="A284" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B284" t="s">
+        <v>521</v>
+      </c>
+      <c r="C284" t="s">
+        <v>31</v>
+      </c>
+      <c r="D284" t="n">
+        <v>258.949263103803</v>
+      </c>
+      <c r="E284" t="n">
+        <v>63</v>
+      </c>
+      <c r="F284" t="n">
+        <v>0</v>
+      </c>
+      <c r="G284" t="n">
+        <v>576</v>
+      </c>
+      <c r="H284" t="n">
+        <v>166</v>
+      </c>
+      <c r="I284" t="n">
+        <v>410</v>
+      </c>
+      <c r="J284" t="n">
+        <v>5</v>
+      </c>
+      <c r="K284" t="n">
+        <v>8649</v>
+      </c>
+      <c r="L284" t="n">
+        <v>29</v>
+      </c>
+      <c r="M284" t="s">
+        <v>522</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-07]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="526">
   <si>
     <t>date</t>
   </si>
@@ -1590,6 +1590,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/chile/liga-de-ascenso/, /football/ecuador/serie-b/, /football/el-salvador/primera-division/, /football/ireland/division-1/, /football/latvia/virsliga/, /football/romania/liga-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">df75fd32d4876a294e57fca3a89d8a7e1476cf0f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/chile/liga-de-ascenso/, /football/colombia/primera-b/, /football/ecuador/serie-b/, /football/el-salvador/primera-division/, /football/finland/ykkosliiga/, /football/guatemala/liga-nacional/, /football/iraq/stars-league/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/paraguay/copa-de-primera/</t>
   </si>
 </sst>
 </file>
@@ -13580,6 +13586,47 @@
         <v>524</v>
       </c>
     </row>
+    <row r="286">
+      <c r="A286" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B286" t="s">
+        <v>525</v>
+      </c>
+      <c r="C286" t="s">
+        <v>31</v>
+      </c>
+      <c r="D286" t="n">
+        <v>304.03647326231</v>
+      </c>
+      <c r="E286" t="n">
+        <v>65</v>
+      </c>
+      <c r="F286" t="n">
+        <v>0</v>
+      </c>
+      <c r="G286" t="n">
+        <v>583</v>
+      </c>
+      <c r="H286" t="n">
+        <v>131</v>
+      </c>
+      <c r="I286" t="n">
+        <v>452</v>
+      </c>
+      <c r="J286" t="n">
+        <v>1</v>
+      </c>
+      <c r="K286" t="n">
+        <v>8853</v>
+      </c>
+      <c r="L286" t="n">
+        <v>25</v>
+      </c>
+      <c r="M286" t="s">
+        <v>526</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-08]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="528">
   <si>
     <t>date</t>
   </si>
@@ -1596,6 +1596,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/chile/liga-de-ascenso/, /football/colombia/primera-b/, /football/ecuador/serie-b/, /football/el-salvador/primera-division/, /football/finland/ykkosliiga/, /football/guatemala/liga-nacional/, /football/iraq/stars-league/, /football/ireland/division-1/, /football/kazakhstan/premier-league/, /football/paraguay/copa-de-primera/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">342e5fbb19c41df4dfac83153f56659cb119f1b6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/canada/canadian-premier-league/, /football/chile/liga-de-ascenso/, /football/costa-rica/liga-de-ascenso/, /football/ecuador/serie-b/, /football/el-salvador/primera-division/, /football/guatemala/liga-nacional/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/mexico/liga-mx/, /football/paraguay/copa-de-primera/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -13627,6 +13633,47 @@
         <v>526</v>
       </c>
     </row>
+    <row r="287">
+      <c r="A287" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B287" t="s">
+        <v>527</v>
+      </c>
+      <c r="C287" t="s">
+        <v>31</v>
+      </c>
+      <c r="D287" t="n">
+        <v>276.544321238995</v>
+      </c>
+      <c r="E287" t="n">
+        <v>69</v>
+      </c>
+      <c r="F287" t="n">
+        <v>0</v>
+      </c>
+      <c r="G287" t="n">
+        <v>610</v>
+      </c>
+      <c r="H287" t="n">
+        <v>138</v>
+      </c>
+      <c r="I287" t="n">
+        <v>472</v>
+      </c>
+      <c r="J287" t="n">
+        <v>7</v>
+      </c>
+      <c r="K287" t="n">
+        <v>9210</v>
+      </c>
+      <c r="L287" t="n">
+        <v>31</v>
+      </c>
+      <c r="M287" t="s">
+        <v>528</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-09]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="532">
   <si>
     <t>date</t>
   </si>
@@ -1608,6 +1608,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/costa-rica/liga-de-ascenso/, /football/croatia/hnl/, /football/el-salvador/primera-division/, /football/estonia/esiliiga/, /football/finland/ykkosliiga/, /football/honduras/liga-nacional/, /football/kazakhstan/premier-league/, /football/malawi/super-league/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3493b4aa0034bce071a798a127d03d60ceddb1c8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/estonia/esiliiga/, /football/guatemala/liga-nacional/, /football/lithuania/i-lyga/, /football/luxembourg/bgl-ligue/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -13721,6 +13727,47 @@
         <v>530</v>
       </c>
     </row>
+    <row r="289">
+      <c r="A289" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B289" t="s">
+        <v>531</v>
+      </c>
+      <c r="C289" t="s">
+        <v>31</v>
+      </c>
+      <c r="D289" t="n">
+        <v>226.520233420531</v>
+      </c>
+      <c r="E289" t="n">
+        <v>76</v>
+      </c>
+      <c r="F289" t="n">
+        <v>0</v>
+      </c>
+      <c r="G289" t="n">
+        <v>646</v>
+      </c>
+      <c r="H289" t="n">
+        <v>198</v>
+      </c>
+      <c r="I289" t="n">
+        <v>448</v>
+      </c>
+      <c r="J289" t="n">
+        <v>5</v>
+      </c>
+      <c r="K289" t="n">
+        <v>9583</v>
+      </c>
+      <c r="L289" t="n">
+        <v>34</v>
+      </c>
+      <c r="M289" t="s">
+        <v>532</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-10]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="536">
   <si>
     <t>date</t>
   </si>
@@ -1620,6 +1620,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/colombia/primera-a/, /football/ethiopia/premier-league/, /football/finland/ykkosliiga/, /football/paraguay/copa-de-primera/, /football/paraguay/division-intermedia/, /football/peru/liga-2/, /football/uzbekistan/super-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">700f47729ad9e3df90012677c7a050de540cedd6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/bulgaria/vtora-liga/, /football/georgia/crystalbet-erovnuli-liga/, /football/ireland/division-1/, /football/malawi/super-league/, /football/paraguay/copa-de-primera/, /football/paraguay/division-intermedia/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -13815,6 +13821,47 @@
         <v>534</v>
       </c>
     </row>
+    <row r="291">
+      <c r="A291" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B291" t="s">
+        <v>535</v>
+      </c>
+      <c r="C291" t="s">
+        <v>31</v>
+      </c>
+      <c r="D291" t="n">
+        <v>315.523983764648</v>
+      </c>
+      <c r="E291" t="n">
+        <v>80</v>
+      </c>
+      <c r="F291" t="n">
+        <v>0</v>
+      </c>
+      <c r="G291" t="n">
+        <v>640</v>
+      </c>
+      <c r="H291" t="n">
+        <v>238</v>
+      </c>
+      <c r="I291" t="n">
+        <v>402</v>
+      </c>
+      <c r="J291" t="n">
+        <v>46</v>
+      </c>
+      <c r="K291" t="n">
+        <v>10202</v>
+      </c>
+      <c r="L291" t="n">
+        <v>33</v>
+      </c>
+      <c r="M291" t="s">
+        <v>536</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-12]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="538">
   <si>
     <t>date</t>
   </si>
@@ -1626,6 +1626,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/bulgaria/vtora-liga/, /football/georgia/crystalbet-erovnuli-liga/, /football/ireland/division-1/, /football/malawi/super-league/, /football/paraguay/copa-de-primera/, /football/paraguay/division-intermedia/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0a73c88982f1e25c098077d09ca2d71e3169e90f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/argentina/primera-nacional/, /football/austria/2-liga/, /football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/ireland/division-1/, /football/lithuania/i-lyga/, /football/turkey/super-lig/</t>
   </si>
 </sst>
 </file>
@@ -13862,6 +13868,47 @@
         <v>536</v>
       </c>
     </row>
+    <row r="292">
+      <c r="A292" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B292" t="s">
+        <v>537</v>
+      </c>
+      <c r="C292" t="s">
+        <v>31</v>
+      </c>
+      <c r="D292" t="n">
+        <v>304.031878451506</v>
+      </c>
+      <c r="E292" t="n">
+        <v>85</v>
+      </c>
+      <c r="F292" t="n">
+        <v>0</v>
+      </c>
+      <c r="G292" t="n">
+        <v>739</v>
+      </c>
+      <c r="H292" t="n">
+        <v>355</v>
+      </c>
+      <c r="I292" t="n">
+        <v>384</v>
+      </c>
+      <c r="J292" t="n">
+        <v>305</v>
+      </c>
+      <c r="K292" t="n">
+        <v>11999</v>
+      </c>
+      <c r="L292" t="n">
+        <v>44</v>
+      </c>
+      <c r="M292" t="s">
+        <v>538</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-13]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="542">
   <si>
     <t>date</t>
   </si>
@@ -1638,6 +1638,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/colombia/primera-a/, /football/colombia/primera-a/, /football/colombia/primera-b/, /football/kazakhstan/premier-league/, /football/romania/superliga/, /football/uruguay/liga-auf-uruguaya/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ca05e17fca12a572a564907fb3c0c853d6f4d681</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/finland/ykkosliiga/, /football/guatemala/liga-nacional/, /football/iraq/stars-league/, /football/kazakhstan/premier-league/, /football/lithuania/i-lyga/, /football/romania/liga-2/</t>
   </si>
 </sst>
 </file>
@@ -13956,6 +13962,47 @@
         <v>540</v>
       </c>
     </row>
+    <row r="294">
+      <c r="A294" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B294" t="s">
+        <v>541</v>
+      </c>
+      <c r="C294" t="s">
+        <v>31</v>
+      </c>
+      <c r="D294" t="n">
+        <v>259.581395077705</v>
+      </c>
+      <c r="E294" t="n">
+        <v>59</v>
+      </c>
+      <c r="F294" t="n">
+        <v>0</v>
+      </c>
+      <c r="G294" t="n">
+        <v>513</v>
+      </c>
+      <c r="H294" t="n">
+        <v>230</v>
+      </c>
+      <c r="I294" t="n">
+        <v>283</v>
+      </c>
+      <c r="J294" t="n">
+        <v>40</v>
+      </c>
+      <c r="K294" t="n">
+        <v>8520</v>
+      </c>
+      <c r="L294" t="n">
+        <v>31</v>
+      </c>
+      <c r="M294" t="s">
+        <v>542</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-14]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="544">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="546">
   <si>
     <t>date</t>
   </si>
@@ -1650,6 +1650,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/colombia/primera-b/, /football/finland/ykkosliiga/, /football/iraq/stars-league/, /football/ireland/division-1/, /football/paraguay/copa-de-primera/, /football/romania/liga-2/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3c9a5cb3d5dc560d156b79ad56a531675c6f107e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/colombia/primera-b/, /football/finland/ykkosliiga/, /football/iraq/stars-league/, /football/kazakhstan/premier-league/, /football/lithuania/i-lyga/, /football/romania/liga-2/, /football/south-america/copa-sudamericana/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -14050,6 +14056,47 @@
         <v>544</v>
       </c>
     </row>
+    <row r="296">
+      <c r="A296" s="1" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B296" t="s">
+        <v>545</v>
+      </c>
+      <c r="C296" t="s">
+        <v>31</v>
+      </c>
+      <c r="D296" t="n">
+        <v>302.271430699031</v>
+      </c>
+      <c r="E296" t="n">
+        <v>65</v>
+      </c>
+      <c r="F296" t="n">
+        <v>0</v>
+      </c>
+      <c r="G296" t="n">
+        <v>580</v>
+      </c>
+      <c r="H296" t="n">
+        <v>233</v>
+      </c>
+      <c r="I296" t="n">
+        <v>347</v>
+      </c>
+      <c r="J296" t="n">
+        <v>11</v>
+      </c>
+      <c r="K296" t="n">
+        <v>9440</v>
+      </c>
+      <c r="L296" t="n">
+        <v>32</v>
+      </c>
+      <c r="M296" t="s">
+        <v>546</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-15]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="548">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="550">
   <si>
     <t>date</t>
   </si>
@@ -1662,6 +1662,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/chile/liga-de-ascenso/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/luxembourg/bgl-ligue/, /football/paraguay/copa-de-primera/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4ebf0053af585c84eb3b122131bd3f1e19355310</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/armenia/premier-league/, /football/belarus/vysshaya-liga/, /football/belgium/jupiler-pro-league/, /football/bulgaria/vtora-liga/, /football/canada/canadian-premier-league/, /football/chile/liga-de-primera/, /football/costa-rica/liga-de-ascenso/, /football/el-salvador/primera-division/, /football/iraq/stars-league/, /football/luxembourg/bgl-ligue/, /football/mexico/liga-mx/, /football/paraguay/copa-de-primera/</t>
   </si>
 </sst>
 </file>
@@ -14144,6 +14150,47 @@
         <v>548</v>
       </c>
     </row>
+    <row r="298">
+      <c r="A298" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B298" t="s">
+        <v>549</v>
+      </c>
+      <c r="C298" t="s">
+        <v>31</v>
+      </c>
+      <c r="D298" t="n">
+        <v>297.508228536447</v>
+      </c>
+      <c r="E298" t="n">
+        <v>73</v>
+      </c>
+      <c r="F298" t="n">
+        <v>0</v>
+      </c>
+      <c r="G298" t="n">
+        <v>592</v>
+      </c>
+      <c r="H298" t="n">
+        <v>234</v>
+      </c>
+      <c r="I298" t="n">
+        <v>358</v>
+      </c>
+      <c r="J298" t="n">
+        <v>28</v>
+      </c>
+      <c r="K298" t="n">
+        <v>10087</v>
+      </c>
+      <c r="L298" t="n">
+        <v>35</v>
+      </c>
+      <c r="M298" t="s">
+        <v>550</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-16]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="554">
   <si>
     <t>date</t>
   </si>
@@ -1674,6 +1674,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/chile/liga-de-ascenso/, /football/ethiopia/premier-league/, /football/finland/ykkosliiga/, /football/honduras/liga-nacional/, /football/lithuania/i-lyga/, /football/luxembourg/bgl-ligue/, /football/paraguay/copa-de-primera/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">55b9acb29056bffc70740c1af226059c02fa91ad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/chile/liga-de-ascenso/, /football/costa-rica/liga-de-ascenso/, /football/georgia/crystalbet-erovnuli-liga/, /football/guatemala/liga-nacional/, /football/luxembourg/bgl-ligue/, /football/mexico/liga-mx/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -14238,6 +14244,47 @@
         <v>552</v>
       </c>
     </row>
+    <row r="300">
+      <c r="A300" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B300" t="s">
+        <v>553</v>
+      </c>
+      <c r="C300" t="s">
+        <v>31</v>
+      </c>
+      <c r="D300" t="n">
+        <v>295.552980569998</v>
+      </c>
+      <c r="E300" t="n">
+        <v>77</v>
+      </c>
+      <c r="F300" t="n">
+        <v>0</v>
+      </c>
+      <c r="G300" t="n">
+        <v>608</v>
+      </c>
+      <c r="H300" t="n">
+        <v>224</v>
+      </c>
+      <c r="I300" t="n">
+        <v>384</v>
+      </c>
+      <c r="J300" t="n">
+        <v>7</v>
+      </c>
+      <c r="K300" t="n">
+        <v>9881</v>
+      </c>
+      <c r="L300" t="n">
+        <v>41</v>
+      </c>
+      <c r="M300" t="s">
+        <v>554</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-17]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="554">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="556">
   <si>
     <t>date</t>
   </si>
@@ -1680,6 +1680,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/chile/liga-de-ascenso/, /football/costa-rica/liga-de-ascenso/, /football/georgia/crystalbet-erovnuli-liga/, /football/guatemala/liga-nacional/, /football/luxembourg/bgl-ligue/, /football/mexico/liga-mx/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4aa6d2d6daad20a31e286439c9dd726afb9b5f4f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/bulgaria/vtora-liga/, /football/costa-rica/liga-de-ascenso/, /football/estonia/esiliiga/, /football/finland/ykkosliiga/, /football/guatemala/liga-nacional/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -14285,6 +14291,47 @@
         <v>554</v>
       </c>
     </row>
+    <row r="301">
+      <c r="A301" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B301" t="s">
+        <v>555</v>
+      </c>
+      <c r="C301" t="s">
+        <v>31</v>
+      </c>
+      <c r="D301" t="n">
+        <v>316.90015788873</v>
+      </c>
+      <c r="E301" t="n">
+        <v>77</v>
+      </c>
+      <c r="F301" t="n">
+        <v>0</v>
+      </c>
+      <c r="G301" t="n">
+        <v>592</v>
+      </c>
+      <c r="H301" t="n">
+        <v>311</v>
+      </c>
+      <c r="I301" t="n">
+        <v>281</v>
+      </c>
+      <c r="J301" t="n">
+        <v>44</v>
+      </c>
+      <c r="K301" t="n">
+        <v>10236</v>
+      </c>
+      <c r="L301" t="n">
+        <v>44</v>
+      </c>
+      <c r="M301" t="s">
+        <v>556</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-18]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="558">
   <si>
     <t>date</t>
   </si>
@@ -1686,6 +1686,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/bulgaria/vtora-liga/, /football/costa-rica/liga-de-ascenso/, /football/estonia/esiliiga/, /football/finland/ykkosliiga/, /football/guatemala/liga-nacional/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">902ebefbd542c87109c58dbb6a9ea71c324c5d90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/austria/2-liga/, /football/belgium/challenger-pro-league/, /football/bulgaria/vtora-liga/, /football/colombia/primera-a/, /football/estonia/esiliiga/, /football/honduras/liga-nacional/, /football/paraguay/division-intermedia/, /football/romania/liga-2/</t>
   </si>
 </sst>
 </file>
@@ -14332,6 +14338,47 @@
         <v>556</v>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B302" t="s">
+        <v>557</v>
+      </c>
+      <c r="C302" t="s">
+        <v>31</v>
+      </c>
+      <c r="D302" t="n">
+        <v>286.854377098878</v>
+      </c>
+      <c r="E302" t="n">
+        <v>90</v>
+      </c>
+      <c r="F302" t="n">
+        <v>0</v>
+      </c>
+      <c r="G302" t="n">
+        <v>594</v>
+      </c>
+      <c r="H302" t="n">
+        <v>321</v>
+      </c>
+      <c r="I302" t="n">
+        <v>273</v>
+      </c>
+      <c r="J302" t="n">
+        <v>161</v>
+      </c>
+      <c r="K302" t="n">
+        <v>12058</v>
+      </c>
+      <c r="L302" t="n">
+        <v>45</v>
+      </c>
+      <c r="M302" t="s">
+        <v>558</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-19]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="562">
   <si>
     <t>date</t>
   </si>
@@ -1698,6 +1698,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/algeria/ligue-1/, /football/austria/2-liga/, /football/belgium/challenger-pro-league/, /football/bulgaria/vtora-liga/, /football/chile/liga-de-primera/, /football/colombia/primera-a/, /football/poland/division-1/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c04ace12d26cefd74185fcbcc5c236aa336d609c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/belgium/challenger-pro-league/, /football/bulgaria/vtora-liga/, /football/colombia/primera-a/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/poland/division-1/</t>
   </si>
 </sst>
 </file>
@@ -14426,6 +14432,47 @@
         <v>560</v>
       </c>
     </row>
+    <row r="304">
+      <c r="A304" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B304" t="s">
+        <v>561</v>
+      </c>
+      <c r="C304" t="s">
+        <v>31</v>
+      </c>
+      <c r="D304" t="n">
+        <v>337.263296612104</v>
+      </c>
+      <c r="E304" t="n">
+        <v>65</v>
+      </c>
+      <c r="F304" t="n">
+        <v>0</v>
+      </c>
+      <c r="G304" t="n">
+        <v>548</v>
+      </c>
+      <c r="H304" t="n">
+        <v>235</v>
+      </c>
+      <c r="I304" t="n">
+        <v>313</v>
+      </c>
+      <c r="J304" t="n">
+        <v>17</v>
+      </c>
+      <c r="K304" t="n">
+        <v>11288</v>
+      </c>
+      <c r="L304" t="n">
+        <v>29</v>
+      </c>
+      <c r="M304" t="s">
+        <v>562</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-20]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="562">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="564">
   <si>
     <t>date</t>
   </si>
@@ -1704,6 +1704,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/belgium/challenger-pro-league/, /football/bulgaria/vtora-liga/, /football/colombia/primera-a/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/poland/division-1/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7c69d6634aee975e4b2a994224b953deabe2195e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/belgium/challenger-pro-league/, /football/chile/liga-de-ascenso/, /football/iraq/stars-league/, /football/lithuania/i-lyga/, /football/poland/division-1/</t>
   </si>
 </sst>
 </file>
@@ -14473,6 +14479,47 @@
         <v>562</v>
       </c>
     </row>
+    <row r="305">
+      <c r="A305" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B305" t="s">
+        <v>563</v>
+      </c>
+      <c r="C305" t="s">
+        <v>31</v>
+      </c>
+      <c r="D305" t="n">
+        <v>236.932783615589</v>
+      </c>
+      <c r="E305" t="n">
+        <v>57</v>
+      </c>
+      <c r="F305" t="n">
+        <v>0</v>
+      </c>
+      <c r="G305" t="n">
+        <v>480</v>
+      </c>
+      <c r="H305" t="n">
+        <v>201</v>
+      </c>
+      <c r="I305" t="n">
+        <v>279</v>
+      </c>
+      <c r="J305" t="n">
+        <v>36</v>
+      </c>
+      <c r="K305" t="n">
+        <v>9063</v>
+      </c>
+      <c r="L305" t="n">
+        <v>26</v>
+      </c>
+      <c r="M305" t="s">
+        <v>564</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-21]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="568">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="570">
   <si>
     <t>date</t>
   </si>
@@ -1722,6 +1722,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/belgium/challenger-pro-league/, /football/guatemala/liga-nacional/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/paraguay/copa-de-primera/, /football/slovenia/prva-liga/, /football/turkey/1-lig/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13f9fcfc97d2354d6b1e66a14df472e37ef072c6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/bulgaria/vtora-liga/, /football/costa-rica/liga-de-ascenso/, /football/ethiopia/premier-league/, /football/japan/j1-league/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/mexico/liga-de-expansion-mx/, /football/northern-ireland/nifl-premiership/, /football/romania/liga-2/, /football/ukraine/premier-league/, /football/usa/usl-championship/</t>
   </si>
 </sst>
 </file>
@@ -14614,6 +14620,47 @@
         <v>568</v>
       </c>
     </row>
+    <row r="308">
+      <c r="A308" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B308" t="s">
+        <v>569</v>
+      </c>
+      <c r="C308" t="s">
+        <v>31</v>
+      </c>
+      <c r="D308" t="n">
+        <v>324.479415675004</v>
+      </c>
+      <c r="E308" t="n">
+        <v>59</v>
+      </c>
+      <c r="F308" t="n">
+        <v>0</v>
+      </c>
+      <c r="G308" t="n">
+        <v>490</v>
+      </c>
+      <c r="H308" t="n">
+        <v>142</v>
+      </c>
+      <c r="I308" t="n">
+        <v>348</v>
+      </c>
+      <c r="J308" t="n">
+        <v>10</v>
+      </c>
+      <c r="K308" t="n">
+        <v>8943</v>
+      </c>
+      <c r="L308" t="n">
+        <v>27</v>
+      </c>
+      <c r="M308" t="s">
+        <v>570</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-22]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="572">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="574">
   <si>
     <t>date</t>
   </si>
@@ -1734,6 +1734,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/estonia/meistriliiga/, /football/estonia/esiliiga/, /football/ethiopia/premier-league/, /football/faroe-islands/premier-league/, /football/iraq/stars-league/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/luxembourg/bgl-ligue/, /football/mexico/liga-de-expansion-mx/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">74d3f4e8198c5727d495b5861b98e160a8484948</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/armenia/premier-league/, /football/belarus/vysshaya-liga/, /football/bosnia-and-herzegovina/prva-liga-fbih/, /football/ecuador/serie-b/, /football/el-salvador/primera-division/, /football/estonia/esiliiga/, /football/ethiopia/premier-league/, /football/finland/veikkausliiga/, /football/guatemala/liga-nacional/, /football/iraq/stars-league/, /football/kazakhstan/premier-league/, /football/paraguay/copa-de-primera/, /football/peru/liga-1/, /football/slovenia/prva-liga/, /football/uruguay/segunda-division/, /football/usa/mls/</t>
   </si>
 </sst>
 </file>
@@ -14708,6 +14714,47 @@
         <v>572</v>
       </c>
     </row>
+    <row r="310">
+      <c r="A310" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B310" t="s">
+        <v>573</v>
+      </c>
+      <c r="C310" t="s">
+        <v>31</v>
+      </c>
+      <c r="D310" t="n">
+        <v>337.09237361749</v>
+      </c>
+      <c r="E310" t="n">
+        <v>59</v>
+      </c>
+      <c r="F310" t="n">
+        <v>0</v>
+      </c>
+      <c r="G310" t="n">
+        <v>509</v>
+      </c>
+      <c r="H310" t="n">
+        <v>143</v>
+      </c>
+      <c r="I310" t="n">
+        <v>366</v>
+      </c>
+      <c r="J310" t="n">
+        <v>13</v>
+      </c>
+      <c r="K310" t="n">
+        <v>9086</v>
+      </c>
+      <c r="L310" t="n">
+        <v>27</v>
+      </c>
+      <c r="M310" t="s">
+        <v>574</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-23]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="578">
   <si>
     <t>date</t>
   </si>
@@ -1746,6 +1746,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/ecuador/serie-b/, /football/egypt/premier-league/, /football/el-salvador/primera-division/, /football/estonia/esiliiga/, /football/faroe-islands/premier-league/, /football/finland/veikkausliiga/, /football/guatemala/liga-nacional/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/lithuania/i-lyga/, /football/paraguay/copa-de-primera/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5ca3c1b95ef8e9bca3e073cdc59e3a850dfc9d63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/bulgaria/vtora-liga/, /football/chile/liga-de-ascenso/, /football/colombia/primera-b/, /football/egypt/premier-league/, /football/el-salvador/primera-division/, /football/estonia/esiliiga/, /football/faroe-islands/premier-league/, /football/kazakhstan/premier-league/, /football/luxembourg/bgl-ligue/, /football/panama/lpf/, /football/paraguay/copa-de-primera/, /football/paraguay/division-intermedia/, /football/slovenia/prva-liga/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -14802,6 +14808,47 @@
         <v>576</v>
       </c>
     </row>
+    <row r="312">
+      <c r="A312" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B312" t="s">
+        <v>577</v>
+      </c>
+      <c r="C312" t="s">
+        <v>31</v>
+      </c>
+      <c r="D312" t="n">
+        <v>333.851272837321</v>
+      </c>
+      <c r="E312" t="n">
+        <v>70</v>
+      </c>
+      <c r="F312" t="n">
+        <v>0</v>
+      </c>
+      <c r="G312" t="n">
+        <v>558</v>
+      </c>
+      <c r="H312" t="n">
+        <v>148</v>
+      </c>
+      <c r="I312" t="n">
+        <v>410</v>
+      </c>
+      <c r="J312" t="n">
+        <v>3</v>
+      </c>
+      <c r="K312" t="n">
+        <v>9740</v>
+      </c>
+      <c r="L312" t="n">
+        <v>34</v>
+      </c>
+      <c r="M312" t="s">
+        <v>578</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-24]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="582">
   <si>
     <t>date</t>
   </si>
@@ -1758,6 +1758,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/egypt/premier-league/, /football/estonia/meistriliiga/, /football/estonia/esiliiga/, /football/faroe-islands/premier-league/, /football/ireland/premier-division/, /football/luxembourg/bgl-ligue/, /football/panama/lpf/, /football/romania/superliga/, /football/slovenia/prva-liga/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">74bce7db37d3e559a708959b1885ca46b13e8f09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/cameroon/elite-one/, /football/canada/canadian-premier-league/, /football/chile/liga-de-primera/, /football/china/super-league/, /football/colombia/primera-a/, /football/costa-rica/liga-de-ascenso/, /football/estonia/meistriliiga/, /football/estonia/esiliiga/, /football/faroe-islands/premier-league/, /football/finland/veikkausliiga/, /football/ireland/premier-division/, /football/kazakhstan/premier-league/, /football/moldova/super-liga/, /football/netherlands/eerste-divisie/, /football/paraguay/division-intermedia/, /football/peru/liga-1/</t>
   </si>
 </sst>
 </file>
@@ -14896,6 +14902,47 @@
         <v>580</v>
       </c>
     </row>
+    <row r="314">
+      <c r="A314" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B314" t="s">
+        <v>581</v>
+      </c>
+      <c r="C314" t="s">
+        <v>31</v>
+      </c>
+      <c r="D314" t="n">
+        <v>300.327722215652</v>
+      </c>
+      <c r="E314" t="n">
+        <v>72</v>
+      </c>
+      <c r="F314" t="n">
+        <v>0</v>
+      </c>
+      <c r="G314" t="n">
+        <v>486</v>
+      </c>
+      <c r="H314" t="n">
+        <v>148</v>
+      </c>
+      <c r="I314" t="n">
+        <v>338</v>
+      </c>
+      <c r="J314" t="n">
+        <v>32</v>
+      </c>
+      <c r="K314" t="n">
+        <v>9531</v>
+      </c>
+      <c r="L314" t="n">
+        <v>33</v>
+      </c>
+      <c r="M314" t="s">
+        <v>582</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-25]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="586">
   <si>
     <t>date</t>
   </si>
@@ -1770,6 +1770,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/algeria/ligue-1/, /football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/chile/liga-de-primera/, /football/denmark/1st-division/, /football/ecuador/serie-b/, /football/egypt/premier-league/, /football/france/ligue-2/, /football/lithuania/i-lyga/, /football/northern-ireland/nifl-premiership/, /football/northern-ireland/nifl-premiership/, /football/paraguay/copa-de-primera/, /football/poland/ekstraklasa/, /football/romania/superliga/, /football/slovenia/prva-liga/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bd40524730be50d1c4cd3399503a12e72f20c79a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/chile/liga-de-primera/, /football/colombia/primera-a/, /football/denmark/1st-division/, /football/egypt/premier-league/, /football/france/ligue-2/, /football/guatemala/liga-nacional/, /football/netherlands/eerste-divisie/, /football/northern-ireland/nifl-premiership/, /football/norway/eliteserien/, /football/panama/lpf/, /football/paraguay/copa-de-primera/, /football/paraguay/division-intermedia/, /football/poland/ekstraklasa/, /football/portugal/liga-portugal-2/, /football/ukraine/premier-league/, /football/uruguay/liga-auf-uruguaya/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -14990,6 +14996,47 @@
         <v>584</v>
       </c>
     </row>
+    <row r="316">
+      <c r="A316" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B316" t="s">
+        <v>585</v>
+      </c>
+      <c r="C316" t="s">
+        <v>31</v>
+      </c>
+      <c r="D316" t="n">
+        <v>340.554086232185</v>
+      </c>
+      <c r="E316" t="n">
+        <v>67</v>
+      </c>
+      <c r="F316" t="n">
+        <v>0</v>
+      </c>
+      <c r="G316" t="n">
+        <v>408</v>
+      </c>
+      <c r="H316" t="n">
+        <v>126</v>
+      </c>
+      <c r="I316" t="n">
+        <v>282</v>
+      </c>
+      <c r="J316" t="n">
+        <v>54</v>
+      </c>
+      <c r="K316" t="n">
+        <v>10061</v>
+      </c>
+      <c r="L316" t="n">
+        <v>25</v>
+      </c>
+      <c r="M316" t="s">
+        <v>586</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-28]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="586">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="588">
   <si>
     <t>date</t>
   </si>
@@ -1776,6 +1776,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/pershaya-liga/, /football/chile/liga-de-primera/, /football/colombia/primera-a/, /football/denmark/1st-division/, /football/egypt/premier-league/, /football/france/ligue-2/, /football/guatemala/liga-nacional/, /football/netherlands/eerste-divisie/, /football/northern-ireland/nifl-premiership/, /football/norway/eliteserien/, /football/panama/lpf/, /football/paraguay/copa-de-primera/, /football/paraguay/division-intermedia/, /football/poland/ekstraklasa/, /football/portugal/liga-portugal-2/, /football/ukraine/premier-league/, /football/uruguay/liga-auf-uruguaya/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33d6ae717515cf24de3b9f856889742149f5b734</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/armenia/premier-league/, /football/austria/2-liga/, /football/belarus/vysshaya-liga/, /football/bolivia/division-profesional/, /football/bosnia-and-herzegovina/prva-liga-fbih/, /football/estonia/meistriliiga/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/luxembourg/bgl-ligue/, /football/mexico/liga-de-expansion-mx/, /football/paraguay/copa-de-primera/, /football/peru/liga-1/, /football/ukraine/premier-league/, /football/usa/mls/</t>
   </si>
 </sst>
 </file>
@@ -15037,6 +15043,47 @@
         <v>586</v>
       </c>
     </row>
+    <row r="317">
+      <c r="A317" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B317" t="s">
+        <v>587</v>
+      </c>
+      <c r="C317" t="s">
+        <v>31</v>
+      </c>
+      <c r="D317" t="n">
+        <v>335.050629727046</v>
+      </c>
+      <c r="E317" t="n">
+        <v>64</v>
+      </c>
+      <c r="F317" t="n">
+        <v>0</v>
+      </c>
+      <c r="G317" t="n">
+        <v>532</v>
+      </c>
+      <c r="H317" t="n">
+        <v>392</v>
+      </c>
+      <c r="I317" t="n">
+        <v>140</v>
+      </c>
+      <c r="J317" t="n">
+        <v>154</v>
+      </c>
+      <c r="K317" t="n">
+        <v>10672</v>
+      </c>
+      <c r="L317" t="n">
+        <v>29</v>
+      </c>
+      <c r="M317" t="s">
+        <v>588</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-29]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="592">
   <si>
     <t>date</t>
   </si>
@@ -1788,6 +1788,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/bolivia/division-profesional/, /football/chile/liga-de-ascenso/, /football/china/super-league/, /football/honduras/liga-nacional/, /football/iraq/stars-league/, /football/kazakhstan/premier-league/, /football/kazakhstan/premier-league/, /football/ukraine/premier-league/, /football/uruguay/segunda-division/, /football/usa/mls/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d0e85cc801351d17f2b2fcf2cfecef6b359d7ceb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/armenia/premier-league/, /football/chile/liga-de-ascenso/, /football/colombia/primera-a/, /football/el-salvador/primera-division/, /football/finland/veikkausliiga/, /football/kazakhstan/premier-league/, /football/latvia/virsliga/, /football/luxembourg/bgl-ligue/, /football/paraguay/copa-de-primera/, /football/peru/liga-1/, /football/romania/liga-2/, /football/ukraine/premier-league/, /football/usa/mls/</t>
   </si>
 </sst>
 </file>
@@ -15131,6 +15137,47 @@
         <v>590</v>
       </c>
     </row>
+    <row r="319">
+      <c r="A319" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B319" t="s">
+        <v>591</v>
+      </c>
+      <c r="C319" t="s">
+        <v>31</v>
+      </c>
+      <c r="D319" t="n">
+        <v>324.991642359893</v>
+      </c>
+      <c r="E319" t="n">
+        <v>61</v>
+      </c>
+      <c r="F319" t="n">
+        <v>0</v>
+      </c>
+      <c r="G319" t="n">
+        <v>501</v>
+      </c>
+      <c r="H319" t="n">
+        <v>237</v>
+      </c>
+      <c r="I319" t="n">
+        <v>264</v>
+      </c>
+      <c r="J319" t="n">
+        <v>21</v>
+      </c>
+      <c r="K319" t="n">
+        <v>9851</v>
+      </c>
+      <c r="L319" t="n">
+        <v>30</v>
+      </c>
+      <c r="M319" t="s">
+        <v>592</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-30]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="596">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="598">
   <si>
     <t>date</t>
   </si>
@@ -1806,6 +1806,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/armenia/premier-league/, /football/iraq/stars-league/, /football/kazakhstan/premier-league/, /football/luxembourg/bgl-ligue/, /football/ukraine/premier-league/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8a3da0a11eebb5133e95da0deac5859472beb7ca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/armenia/premier-league/, /football/belarus/vysshaya-liga/, /football/belarus/pershaya-liga/, /football/bulgaria/vtora-liga/, /football/el-salvador/primera-division/, /football/estonia/esiliiga/, /football/georgia/crystalbet-erovnuli-liga/, /football/guatemala/liga-nacional/, /football/luxembourg/bgl-ligue/, /football/paraguay/copa-de-primera/, /football/peru/liga-2/, /football/poland/ekstraklasa/, /football/uruguay/segunda-division/</t>
   </si>
 </sst>
 </file>
@@ -15272,6 +15278,47 @@
         <v>596</v>
       </c>
     </row>
+    <row r="322">
+      <c r="A322" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B322" t="s">
+        <v>597</v>
+      </c>
+      <c r="C322" t="s">
+        <v>31</v>
+      </c>
+      <c r="D322" t="n">
+        <v>270.814545528094</v>
+      </c>
+      <c r="E322" t="n">
+        <v>70</v>
+      </c>
+      <c r="F322" t="n">
+        <v>0</v>
+      </c>
+      <c r="G322" t="n">
+        <v>544</v>
+      </c>
+      <c r="H322" t="n">
+        <v>165</v>
+      </c>
+      <c r="I322" t="n">
+        <v>379</v>
+      </c>
+      <c r="J322" t="n">
+        <v>11</v>
+      </c>
+      <c r="K322" t="n">
+        <v>10374</v>
+      </c>
+      <c r="L322" t="n">
+        <v>31</v>
+      </c>
+      <c r="M322" t="s">
+        <v>598</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update scraped data [2026-10-31]
</commit_message>
<xml_diff>
--- a/data/log/scraper_log.xlsx
+++ b/data/log/scraper_log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="600">
   <si>
     <t>date</t>
   </si>
@@ -1812,6 +1812,12 @@
   </si>
   <si>
     <t xml:space="preserve">/football/armenia/premier-league/, /football/belarus/vysshaya-liga/, /football/belarus/pershaya-liga/, /football/bulgaria/vtora-liga/, /football/el-salvador/primera-division/, /football/estonia/esiliiga/, /football/georgia/crystalbet-erovnuli-liga/, /football/guatemala/liga-nacional/, /football/luxembourg/bgl-ligue/, /football/paraguay/copa-de-primera/, /football/peru/liga-2/, /football/poland/ekstraklasa/, /football/uruguay/segunda-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d43baff49a067ddf1261b4c3e8b40d44c3ea2784</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/football/belarus/vysshaya-liga/, /football/belarus/pershaya-liga/, /football/colombia/primera-a/, /football/el-salvador/primera-division/, /football/estonia/esiliiga/, /football/georgia/crystalbet-erovnuli-liga/, /football/guatemala/liga-nacional/, /football/peru/liga-2/, /football/romania/superliga/</t>
   </si>
 </sst>
 </file>
@@ -15319,6 +15325,47 @@
         <v>598</v>
       </c>
     </row>
+    <row r="323">
+      <c r="A323" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B323" t="s">
+        <v>599</v>
+      </c>
+      <c r="C323" t="s">
+        <v>31</v>
+      </c>
+      <c r="D323" t="n">
+        <v>294.055830260118</v>
+      </c>
+      <c r="E323" t="n">
+        <v>77</v>
+      </c>
+      <c r="F323" t="n">
+        <v>0</v>
+      </c>
+      <c r="G323" t="n">
+        <v>573</v>
+      </c>
+      <c r="H323" t="n">
+        <v>242</v>
+      </c>
+      <c r="I323" t="n">
+        <v>331</v>
+      </c>
+      <c r="J323" t="n">
+        <v>23</v>
+      </c>
+      <c r="K323" t="n">
+        <v>11068</v>
+      </c>
+      <c r="L323" t="n">
+        <v>31</v>
+      </c>
+      <c r="M323" t="s">
+        <v>600</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>